<commit_message>
Revisión de coincidencias comisión 6, 45/118 por el momento
</commit_message>
<xml_diff>
--- a/coincidencias_comisiones.xlsx
+++ b/coincidencias_comisiones.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/044771503088af63/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vicel\Proyectos\constitutional-proposal-tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="685" documentId="8_{4C345CB1-7C1D-49F0-8F7F-9A802A662A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A2AE0F0-A710-4C4C-AE53-83882820C48F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E3189F-B805-41F1-97BD-EAF034DA85AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="10980" windowHeight="13770" activeTab="1" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="2" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
   </bookViews>
   <sheets>
     <sheet name="Comisión 1" sheetId="1" r:id="rId1"/>
     <sheet name="Comisión 3" sheetId="2" r:id="rId2"/>
+    <sheet name="Comisión 6" sheetId="3" r:id="rId3"/>
+    <sheet name="Comisión 5" sheetId="4" r:id="rId4"/>
+    <sheet name="Comisión 7" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comisión 1'!$A$1:$G$1</definedName>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="269">
   <si>
     <t>Número previo</t>
   </si>
@@ -704,13 +707,157 @@
   </si>
   <si>
     <t>C3-GEN-CH01-ART29</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART1</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART2</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART4</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART5</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART6</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART7</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART9</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART10</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART11</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART12</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART15</t>
+  </si>
+  <si>
+    <t>Una palabra de diferencia</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART18</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART18A</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART21</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART22</t>
+  </si>
+  <si>
+    <t>C6_IND02-08_ART16</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART24</t>
+  </si>
+  <si>
+    <t>Sobra un inciso</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART25</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART3</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART4</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART5</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART6</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART7</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART29</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART9</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART30</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART34</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART37</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART41</t>
+  </si>
+  <si>
+    <t>C6_IND03-07_ART16</t>
+  </si>
+  <si>
+    <t>C6_X_ART24</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART45</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART46</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART47</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART48</t>
+  </si>
+  <si>
+    <t>Sobran dos incisos</t>
+  </si>
+  <si>
+    <t>C6_X_ART28B</t>
+  </si>
+  <si>
+    <t>C6_X_ART42</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART64</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART66</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART67</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART69</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART70</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART73</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART74A</t>
+  </si>
+  <si>
+    <t>C6_GEN1_ART77</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,6 +876,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFA31515"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -751,9 +904,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3980,4 +4136,1511 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5520BB1-FD64-4562-8A4D-B7ECF35F2484}">
+  <dimension ref="A1:G120"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>339</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>340</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>341</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>342</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>343</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>344</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>345</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>346</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>347</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>348</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>349</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E12" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>350</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>351</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>352</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>353</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>354</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>355</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E18" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>356</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>357</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>358</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>359</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>360</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>361</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>362</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>363</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>364</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>365</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E28" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>366</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>367</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>368</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>369</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>370</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>371</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>372</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>4</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>373</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E36" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>374</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>375</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>376</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>377</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>378</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>379</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>4</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>380</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>4</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>381</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>4</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>382</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>4</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>383</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>384</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>385</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>386</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>387</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>388</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>389</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>390</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>391</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>392</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>393</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>394</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>395</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>396</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>397</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>398</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>399</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>400</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>401</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>402</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>403</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>404</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>405</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>406</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>407</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>408</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>409</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>410</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>411</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>412</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>413</v>
+      </c>
+      <c r="B76">
+        <v>1</v>
+      </c>
+      <c r="C76" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>414</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="C77" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>415</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+      <c r="C78" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>416</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>417</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>418</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>419</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83">
+        <v>420</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+      <c r="C83" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>421</v>
+      </c>
+      <c r="B84">
+        <v>1</v>
+      </c>
+      <c r="C84" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85">
+        <v>422</v>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+      <c r="C85" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86">
+        <v>423</v>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+      <c r="C86" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87">
+        <v>424</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>425</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>426</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>427</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>428</v>
+      </c>
+      <c r="B91">
+        <v>1</v>
+      </c>
+      <c r="C91" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>429</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>430</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>431</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>432</v>
+      </c>
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>433</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+      <c r="C96" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>434</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>435</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>436</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+      <c r="C99" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>437</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>438</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>439</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>440</v>
+      </c>
+      <c r="B103">
+        <v>1</v>
+      </c>
+      <c r="C103" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <v>441</v>
+      </c>
+      <c r="B104">
+        <v>1</v>
+      </c>
+      <c r="C104" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <v>442</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <v>443</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <v>444</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <v>445</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <v>446</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <v>447</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <v>448</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <v>449</v>
+      </c>
+      <c r="B112">
+        <v>1</v>
+      </c>
+      <c r="C112" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>450</v>
+      </c>
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>451</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>452</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>453</v>
+      </c>
+      <c r="B116">
+        <v>1</v>
+      </c>
+      <c r="C116" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>454</v>
+      </c>
+      <c r="B117">
+        <v>1</v>
+      </c>
+      <c r="C117" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>455</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>456</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>457</v>
+      </c>
+      <c r="B120">
+        <v>1</v>
+      </c>
+      <c r="C120" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF016F2B-E88B-426D-8061-4E20A3875DD7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C625EF6D-2FED-45E6-AF0C-2B30004BDDFE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
final_status añadido a la comisión 6. Se reportan 100 artículos idénticos al borrador final, 18 similares y 1 perdido por el momento. Está pendiente una revisión manual del historial de los artículos aún no idénticos
</commit_message>
<xml_diff>
--- a/coincidencias_comisiones.xlsx
+++ b/coincidencias_comisiones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vicel\Proyectos\constitutional-proposal-tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E3189F-B805-41F1-97BD-EAF034DA85AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0EA444-BD9F-4C49-A0EC-5EDD919F1D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="2" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
   </bookViews>
@@ -22,6 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comisión 1'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comisión 3'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comisión 6'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="345">
   <si>
     <t>Número previo</t>
   </si>
@@ -851,6 +852,234 @@
   </si>
   <si>
     <t>C6_GEN1_ART77</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART1</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART3</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART8</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART9</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART10</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART10A</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART11</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART13</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART14</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART17</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ART12BIS</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART19</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ART13BIS</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ART13TER</t>
+  </si>
+  <si>
+    <t>C6_IND04-01-2_ART15</t>
+  </si>
+  <si>
+    <t>C6_IND04-01-2_ART16</t>
+  </si>
+  <si>
+    <t>C6_IND04-27_ART17</t>
+  </si>
+  <si>
+    <t>C6_IND04-27_ART18</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART22</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART24</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART25</t>
+  </si>
+  <si>
+    <t>Una coma de diferencia</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART27</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART34</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART36A</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART37</t>
+  </si>
+  <si>
+    <t>C6_IND04-27_ART29</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART41</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART42</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART43</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART56A</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ART35BIS</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART61</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART62</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART62C</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART63A</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART64</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART65C</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART69</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART70</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART73B</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART74</t>
+  </si>
+  <si>
+    <t>"de la Contraloría" sobra</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART75</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART76</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART77</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART78</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART82</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART87</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART88</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART91</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART101</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART89</t>
+  </si>
+  <si>
+    <t>Una letra de diferencia</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART114</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART108</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART116</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART117A</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ART68BIS</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART118A</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART119</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART127</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART129</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART130</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART131</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART136</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART137</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART138</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART140</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART141</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART142</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART145</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART148</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART149</t>
+  </si>
+  <si>
+    <t>C6_GEN3_ART150</t>
+  </si>
+  <si>
+    <t>C6_IND05-08_ARTN90</t>
   </si>
 </sst>
 </file>
@@ -4196,21 +4425,21 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -4219,12 +4448,12 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -4233,12 +4462,12 @@
         <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -4247,12 +4476,12 @@
         <v>4</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -4261,12 +4490,12 @@
         <v>4</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -4275,12 +4504,12 @@
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -4289,12 +4518,12 @@
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -4303,43 +4532,40 @@
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E12" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="E13" t="s">
-        <v>150</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -4348,12 +4574,12 @@
         <v>4</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -4362,12 +4588,12 @@
         <v>4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -4376,12 +4602,12 @@
         <v>4</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -4390,1239 +4616,1502 @@
         <v>4</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
+        <v>359</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>360</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>361</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>362</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>363</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>364</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>366</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>367</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>368</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>369</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>371</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>372</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>374</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>375</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>376</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>377</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>378</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>379</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>4</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>380</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>4</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>381</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>382</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>383</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>384</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>385</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>387</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>4</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>388</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>4</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>389</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>4</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>390</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>4</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>391</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>392</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>4</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>393</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>394</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>4</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>395</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>4</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>396</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>397</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>398</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>399</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>4</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>400</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>401</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>402</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>403</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>4</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>404</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>406</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>4</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>407</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>4</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>408</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>4</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>409</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>410</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
+        <v>4</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>411</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" t="s">
+        <v>4</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>412</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>4</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>413</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>4</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>414</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>4</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>415</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>4</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>416</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>417</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>4</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>418</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>4</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>419</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>4</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>420</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>4</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>421</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>4</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>422</v>
+      </c>
+      <c r="B76">
+        <v>1</v>
+      </c>
+      <c r="C76" t="s">
+        <v>4</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>423</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="C77" t="s">
+        <v>4</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>424</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+      <c r="C78" t="s">
+        <v>4</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>426</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>4</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>427</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>428</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>4</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>429</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>4</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83">
+        <v>431</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+      <c r="C83" t="s">
+        <v>4</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>432</v>
+      </c>
+      <c r="B84">
+        <v>1</v>
+      </c>
+      <c r="C84" t="s">
+        <v>4</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85">
+        <v>435</v>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+      <c r="C85" t="s">
+        <v>4</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86">
+        <v>436</v>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+      <c r="C86" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87">
+        <v>438</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s">
+        <v>4</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>439</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s">
+        <v>4</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>440</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>4</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>442</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>4</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>443</v>
+      </c>
+      <c r="B91">
+        <v>1</v>
+      </c>
+      <c r="C91" t="s">
+        <v>4</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>444</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>4</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>445</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>4</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>446</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>4</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>448</v>
+      </c>
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95" t="s">
+        <v>4</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>450</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+      <c r="C96" t="s">
+        <v>4</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>452</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>4</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>454</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E98" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>455</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+      <c r="C99" t="s">
+        <v>4</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>456</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>4</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>457</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>4</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>341</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>2</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>349</v>
+      </c>
+      <c r="B103">
+        <v>1</v>
+      </c>
+      <c r="C103" t="s">
+        <v>2</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E103" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104">
         <v>355</v>
       </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="B104">
+        <v>1</v>
+      </c>
+      <c r="C104" t="s">
+        <v>2</v>
+      </c>
+      <c r="D104" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E104" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>356</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>357</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>358</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>359</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>360</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <v>361</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>362</v>
-      </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>363</v>
-      </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>364</v>
-      </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105">
         <v>365</v>
       </c>
-      <c r="B28">
-        <v>1</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>2</v>
+      </c>
+      <c r="D105" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E105" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>366</v>
-      </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s">
-        <v>4</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30">
-        <v>367</v>
-      </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
-        <v>4</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31">
-        <v>368</v>
-      </c>
-      <c r="B31">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
-        <v>4</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32">
-        <v>369</v>
-      </c>
-      <c r="B32">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s">
-        <v>4</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A106">
         <v>370</v>
       </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s">
-        <v>2</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>2</v>
+      </c>
+      <c r="D106" s="2" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34">
-        <v>371</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35">
-        <v>372</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>4</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A107">
         <v>373</v>
       </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>2</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>2</v>
+      </c>
+      <c r="D107" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E107" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37">
-        <v>374</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s">
-        <v>4</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38">
-        <v>375</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
-        <v>4</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39">
-        <v>376</v>
-      </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40">
-        <v>377</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
-        <v>4</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41">
-        <v>378</v>
-      </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s">
-        <v>4</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42">
-        <v>379</v>
-      </c>
-      <c r="B42">
-        <v>1</v>
-      </c>
-      <c r="C42" t="s">
-        <v>4</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43">
-        <v>380</v>
-      </c>
-      <c r="B43">
-        <v>1</v>
-      </c>
-      <c r="C43" t="s">
-        <v>4</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44">
-        <v>381</v>
-      </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
-        <v>4</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45">
-        <v>382</v>
-      </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>4</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46">
-        <v>383</v>
-      </c>
-      <c r="B46">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s">
-        <v>4</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47">
-        <v>384</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48">
-        <v>385</v>
-      </c>
-      <c r="B48">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A49">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A108">
         <v>386</v>
       </c>
-      <c r="B49">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50">
-        <v>387</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A51">
-        <v>388</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52">
-        <v>389</v>
-      </c>
-      <c r="B52">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A53">
-        <v>390</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54">
-        <v>391</v>
-      </c>
-      <c r="B54">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55">
-        <v>392</v>
-      </c>
-      <c r="B55">
-        <v>1</v>
-      </c>
-      <c r="C55" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A56">
-        <v>393</v>
-      </c>
-      <c r="B56">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57">
-        <v>394</v>
-      </c>
-      <c r="B57">
-        <v>1</v>
-      </c>
-      <c r="C57" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A58">
-        <v>395</v>
-      </c>
-      <c r="B58">
-        <v>1</v>
-      </c>
-      <c r="C58" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A59">
-        <v>396</v>
-      </c>
-      <c r="B59">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A60">
-        <v>397</v>
-      </c>
-      <c r="B60">
-        <v>1</v>
-      </c>
-      <c r="C60" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61">
-        <v>398</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A62">
-        <v>399</v>
-      </c>
-      <c r="B62">
-        <v>1</v>
-      </c>
-      <c r="C62" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A63">
-        <v>400</v>
-      </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="C63" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A64">
-        <v>401</v>
-      </c>
-      <c r="B64">
-        <v>1</v>
-      </c>
-      <c r="C64" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A65">
-        <v>402</v>
-      </c>
-      <c r="B65">
-        <v>1</v>
-      </c>
-      <c r="C65" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A66">
-        <v>403</v>
-      </c>
-      <c r="B66">
-        <v>1</v>
-      </c>
-      <c r="C66" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A67">
-        <v>404</v>
-      </c>
-      <c r="B67">
-        <v>1</v>
-      </c>
-      <c r="C67" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A68">
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>2</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E108" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A109">
         <v>405</v>
       </c>
-      <c r="B68">
-        <v>1</v>
-      </c>
-      <c r="C68" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A69">
-        <v>406</v>
-      </c>
-      <c r="B69">
-        <v>1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A70">
-        <v>407</v>
-      </c>
-      <c r="B70">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A71">
-        <v>408</v>
-      </c>
-      <c r="B71">
-        <v>1</v>
-      </c>
-      <c r="C71" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A72">
-        <v>409</v>
-      </c>
-      <c r="B72">
-        <v>1</v>
-      </c>
-      <c r="C72" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A73">
-        <v>410</v>
-      </c>
-      <c r="B73">
-        <v>1</v>
-      </c>
-      <c r="C73" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A74">
-        <v>411</v>
-      </c>
-      <c r="B74">
-        <v>1</v>
-      </c>
-      <c r="C74" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A75">
-        <v>412</v>
-      </c>
-      <c r="B75">
-        <v>1</v>
-      </c>
-      <c r="C75" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A76">
-        <v>413</v>
-      </c>
-      <c r="B76">
-        <v>1</v>
-      </c>
-      <c r="C76" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A77">
-        <v>414</v>
-      </c>
-      <c r="B77">
-        <v>1</v>
-      </c>
-      <c r="C77" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A78">
-        <v>415</v>
-      </c>
-      <c r="B78">
-        <v>1</v>
-      </c>
-      <c r="C78" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A79">
-        <v>416</v>
-      </c>
-      <c r="B79">
-        <v>1</v>
-      </c>
-      <c r="C79" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A80">
-        <v>417</v>
-      </c>
-      <c r="B80">
-        <v>1</v>
-      </c>
-      <c r="C80" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A81">
-        <v>418</v>
-      </c>
-      <c r="B81">
-        <v>1</v>
-      </c>
-      <c r="C81" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A82">
-        <v>419</v>
-      </c>
-      <c r="B82">
-        <v>1</v>
-      </c>
-      <c r="C82" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A83">
-        <v>420</v>
-      </c>
-      <c r="B83">
-        <v>1</v>
-      </c>
-      <c r="C83" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A84">
-        <v>421</v>
-      </c>
-      <c r="B84">
-        <v>1</v>
-      </c>
-      <c r="C84" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A85">
-        <v>422</v>
-      </c>
-      <c r="B85">
-        <v>1</v>
-      </c>
-      <c r="C85" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A86">
-        <v>423</v>
-      </c>
-      <c r="B86">
-        <v>1</v>
-      </c>
-      <c r="C86" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A87">
-        <v>424</v>
-      </c>
-      <c r="B87">
-        <v>1</v>
-      </c>
-      <c r="C87" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A88">
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>2</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E109" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A110">
         <v>425</v>
       </c>
-      <c r="B88">
-        <v>1</v>
-      </c>
-      <c r="C88" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A89">
-        <v>426</v>
-      </c>
-      <c r="B89">
-        <v>1</v>
-      </c>
-      <c r="C89" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A90">
-        <v>427</v>
-      </c>
-      <c r="B90">
-        <v>1</v>
-      </c>
-      <c r="C90" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A91">
-        <v>428</v>
-      </c>
-      <c r="B91">
-        <v>1</v>
-      </c>
-      <c r="C91" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A92">
-        <v>429</v>
-      </c>
-      <c r="B92">
-        <v>1</v>
-      </c>
-      <c r="C92" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A93">
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>2</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="E110" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A111">
         <v>430</v>
       </c>
-      <c r="B93">
-        <v>1</v>
-      </c>
-      <c r="C93" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A94">
-        <v>431</v>
-      </c>
-      <c r="B94">
-        <v>1</v>
-      </c>
-      <c r="C94" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A95">
-        <v>432</v>
-      </c>
-      <c r="B95">
-        <v>1</v>
-      </c>
-      <c r="C95" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A96">
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>2</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E111" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A112">
         <v>433</v>
       </c>
-      <c r="B96">
-        <v>1</v>
-      </c>
-      <c r="C96" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A97">
+      <c r="B112">
+        <v>1</v>
+      </c>
+      <c r="C112" t="s">
+        <v>2</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="E112" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A113">
         <v>434</v>
       </c>
-      <c r="B97">
-        <v>1</v>
-      </c>
-      <c r="C97" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A98">
-        <v>435</v>
-      </c>
-      <c r="B98">
-        <v>1</v>
-      </c>
-      <c r="C98" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A99">
-        <v>436</v>
-      </c>
-      <c r="B99">
-        <v>1</v>
-      </c>
-      <c r="C99" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A100">
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113" t="s">
+        <v>2</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E113" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A114">
         <v>437</v>
       </c>
-      <c r="B100">
-        <v>1</v>
-      </c>
-      <c r="C100" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A101">
-        <v>438</v>
-      </c>
-      <c r="B101">
-        <v>1</v>
-      </c>
-      <c r="C101" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A102">
-        <v>439</v>
-      </c>
-      <c r="B102">
-        <v>1</v>
-      </c>
-      <c r="C102" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A103">
-        <v>440</v>
-      </c>
-      <c r="B103">
-        <v>1</v>
-      </c>
-      <c r="C103" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A104">
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>2</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E114" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A115">
         <v>441</v>
       </c>
-      <c r="B104">
-        <v>1</v>
-      </c>
-      <c r="C104" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A105">
-        <v>442</v>
-      </c>
-      <c r="B105">
-        <v>1</v>
-      </c>
-      <c r="C105" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A106">
-        <v>443</v>
-      </c>
-      <c r="B106">
-        <v>1</v>
-      </c>
-      <c r="C106" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A107">
-        <v>444</v>
-      </c>
-      <c r="B107">
-        <v>1</v>
-      </c>
-      <c r="C107" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A108">
-        <v>445</v>
-      </c>
-      <c r="B108">
-        <v>1</v>
-      </c>
-      <c r="C108" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A109">
-        <v>446</v>
-      </c>
-      <c r="B109">
-        <v>1</v>
-      </c>
-      <c r="C109" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A110">
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>2</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E115" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A116">
         <v>447</v>
       </c>
-      <c r="B110">
-        <v>1</v>
-      </c>
-      <c r="C110" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A111">
-        <v>448</v>
-      </c>
-      <c r="B111">
-        <v>1</v>
-      </c>
-      <c r="C111" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A112">
+      <c r="B116">
+        <v>1</v>
+      </c>
+      <c r="C116" t="s">
+        <v>2</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E116" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A117">
         <v>449</v>
       </c>
-      <c r="B112">
-        <v>1</v>
-      </c>
-      <c r="C112" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A113">
-        <v>450</v>
-      </c>
-      <c r="B113">
-        <v>1</v>
-      </c>
-      <c r="C113" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A114">
+      <c r="B117">
+        <v>1</v>
+      </c>
+      <c r="C117" t="s">
+        <v>2</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="E117" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A118">
         <v>451</v>
       </c>
-      <c r="B114">
-        <v>1</v>
-      </c>
-      <c r="C114" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A115">
-        <v>452</v>
-      </c>
-      <c r="B115">
-        <v>1</v>
-      </c>
-      <c r="C115" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A116">
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>2</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A119">
         <v>453</v>
       </c>
-      <c r="B116">
-        <v>1</v>
-      </c>
-      <c r="C116" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A117">
-        <v>454</v>
-      </c>
-      <c r="B117">
-        <v>1</v>
-      </c>
-      <c r="C117" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A118">
-        <v>455</v>
-      </c>
-      <c r="B118">
-        <v>1</v>
-      </c>
-      <c r="C118" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A119">
-        <v>456</v>
-      </c>
       <c r="B119">
         <v>1</v>
       </c>
       <c r="C119" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120">
-        <v>457</v>
+        <v>350</v>
       </c>
       <c r="B120">
-        <v>1</v>
-      </c>
-      <c r="C120" t="s">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E120" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1" xr:uid="{B5520BB1-FD64-4562-8A4D-B7ECF35F2484}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G120">
+      <sortCondition ref="C1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Todos los informes de indicaciones integrados (el último con cierta parcialidad por dificultades en artículos eliminados). Respecto al borrador final, se reportan 25 artículos idénticos y 16 similares
</commit_message>
<xml_diff>
--- a/coincidencias_comisiones.xlsx
+++ b/coincidencias_comisiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vicel\Proyectos\constitutional-proposal-tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0EA444-BD9F-4C49-A0EC-5EDD919F1D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274682E4-40F4-4BC3-B332-8A1DC514EBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="2" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="4" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
   </bookViews>
   <sheets>
     <sheet name="Comisión 1" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comisión 1'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comisión 3'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comisión 6'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Comisión 7'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="388">
   <si>
     <t>Número previo</t>
   </si>
@@ -1080,6 +1081,135 @@
   </si>
   <si>
     <t>C6_IND05-08_ARTN90</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART18</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART20</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART60</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART28</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH1_ART1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH1_ART1_2</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH1_ART3_2</t>
+  </si>
+  <si>
+    <t>C7_GEN2_ART2</t>
+  </si>
+  <si>
+    <t>Un inciso de sobra</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH1_ART4</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH2_ART1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH2_ART3</t>
+  </si>
+  <si>
+    <t>C7_IND03-19_CH13_ART8</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH3_ART1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH3_ART2</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH3_ART2_1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH3_ART2_2</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH3_ART3</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH4_ART1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH5_ARTXX1</t>
+  </si>
+  <si>
+    <t>C7_GEN2_CH6_ARTX</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH01-ART01</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH01-ART01.1</t>
+  </si>
+  <si>
+    <t>C7_IND04-19_ART5</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH04-ART01.1</t>
+  </si>
+  <si>
+    <t>Dos incisos de sobra</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH07-ART15</t>
+  </si>
+  <si>
+    <t>Una palabra</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH08-ART01</t>
+  </si>
+  <si>
+    <t>C7-GEN-CH08-ART01.1</t>
+  </si>
+  <si>
+    <t>C7_IND04-19_ARTN11</t>
+  </si>
+  <si>
+    <t>C7_IND04-19_ARTN3</t>
+  </si>
+  <si>
+    <t>C7_IND03-19_CH11_ART3</t>
+  </si>
+  <si>
+    <t>C7_IND03-19_CH12_ART1</t>
+  </si>
+  <si>
+    <t>C7_IND03-19_CH13_ART6</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART1</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART2</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART6</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART11</t>
+  </si>
+  <si>
+    <t>C7_IND04-09-2_ARTN</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART48</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART50</t>
+  </si>
+  <si>
+    <t>C7_GEN3_ART53</t>
   </si>
 </sst>
 </file>
@@ -6127,9 +6257,648 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C625EF6D-2FED-45E6-AF0C-2B30004BDDFE}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>458</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>459</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>460</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>462</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>464</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>467</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>468</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>469</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>470</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>471</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>472</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>474</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>477</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>480</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>483</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>484</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>485</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>486</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>489</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>490</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>491</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>492</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>493</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>496</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>498</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>461</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E27" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>463</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="E28" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>465</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>466</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>473</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="E31" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>475</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="E32" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>476</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>478</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E34" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>479</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>2</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E35" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>481</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E36" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>482</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E37" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>487</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E38" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>488</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="E39" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>494</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>495</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="E41" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>497</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="E42" t="s">
+        <v>353</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1" xr:uid="{C625EF6D-2FED-45E6-AF0C-2B30004BDDFE}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G42">
+      <sortCondition ref="C1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se dejaron las id únicamente con guión bajo para dejarlas en un formato único
</commit_message>
<xml_diff>
--- a/coincidencias_comisiones.xlsx
+++ b/coincidencias_comisiones.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vicel\Proyectos\constitutional-proposal-tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E811FBC0-36C5-4AD8-AD87-95C95CE040EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B765E9D-078A-40C9-BC8F-8964DEFCD388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="1" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
+    <workbookView xWindow="1900" yWindow="830" windowWidth="17680" windowHeight="12850" xr2:uid="{EB1ABC4A-685D-416C-81A4-F83CAA4FCE57}"/>
   </bookViews>
   <sheets>
     <sheet name="Comisión 1" sheetId="1" r:id="rId1"/>

</xml_diff>